<commit_message>
Expand Espresso coverage and finalize Excel QA reports
</commit_message>
<xml_diff>
--- a/Bugs.xlsx
+++ b/Bugs.xlsx
@@ -142,8 +142,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BugsData" displayName="BugsData" ref="A1:R2" headerRowCount="1">
-  <autoFilter ref="A1:R2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BugsData" displayName="BugsData" ref="A1:R5" headerRowCount="1">
+  <autoFilter ref="A1:R5"/>
   <tableColumns count="18">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Заголовок"/>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -595,7 +595,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Открыт; подтверждён автотестом 22.10.2026</t>
+          <t>Открыт; повторно подтверждён UI-автотестом 26.10.2026</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -634,17 +634,17 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Дата создания соответствует дате создания записи: 21.10.2026 для зафиксированного прогона. При повторном прогоне 22.10.2026 ожидается 22.10.2026.</t>
+          <t>Дата создания соответствует дате создания записи: 21.10.2026 для зафиксированного прогона. При повторном прогоне 22.10.2026 ожидается 22.10.2026. В расширенном прогоне 26.10.2026 ожидается 26.10.2026.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Creation date = 03.01.58775; Publication date = 21.10.2026. Расхождение сохраняется после повторной загрузки панели. Автопрогон 22.10.2026: вместо 22.10.2026 отображается 25.08.58777; NewsRegressionTests.creationDateEqualsToday завершается assertion failure. Ручной прогон 22.10.2026: дата создания 22.08.58777 вместо 22.10.2026. Ошибочная дата меняется между созданиями; дефект — несоответствие реальной дате, а не конкретное постоянное значение.</t>
+          <t>Creation date = 03.01.58775; Publication date = 21.10.2026. Расхождение сохраняется после повторной загрузки панели. Автопрогон 22.10.2026: вместо 22.10.2026 отображается 25.08.58777; NewsRegressionTests.creationDateEqualsToday завершается assertion failure. Предварительный UI-прогон 22.10.2026: дата создания 22.08.58777 вместо 22.10.2026. Ошибочная дата меняется между созданиями; дефект — несоответствие реальной дате, а не конкретное постоянное значение. Полный UI-прогон 26.10.2026: вместо 26.10.2026 отображается 02.04.58789.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Подтверждён при первичной проверке 21.10.2026, повторной проверке интерфейса и UI-автотестом 22.10.2026.</t>
+          <t>Подтверждён при первичной проверке 21.10.2026, повторной проверке интерфейса и UI-автотестом 22.10.2026. Повторно подтверждён в полном прогоне 26.10.2026.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -659,12 +659,289 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>docs/evidence/stage1/own-news-panel.png; docs/evidence/stage1/own-news-open.png; docs/evidence/stage1/own-inactive-location.png; docs/evidence/stage2/BUG-001-creation-date.png; allure-results.zip; docs/evidence/manual-run/creation-date-defect.png; docs/evidence/manual-run/timings.json</t>
+          <t>docs/evidence/stage1/own-news-panel.png; docs/evidence/stage1/own-news-open.png; docs/evidence/stage1/own-inactive-location.png; docs/evidence/stage2/BUG-001-creation-date.png; allure-results.zip; docs/evidence/manual-run/creation-date-defect.png; docs/evidence/manual-run/timings.json; docs/evidence/expanded-2026-10-26/BUG-001-creation-date.png</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Исходная тестовая запись удалена после проверки. Причина на стороне клиента или сервера не установлена.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="360" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>BUG-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Введённый логин не читается в тёмной теме</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Major / значительная</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>P1 / высокий</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Открыт; подтверждён полным UI-прогоном 26.10.2026</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Авторизация / тёмная тема</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>1.0.0 (14), debug</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Android 16 / API 36; x86_64; Pixel 6, 1080×2400; en-US; GMT / UTC; debug 1.0.0 (14); AGP 8.12.2 / Gradle 8.13. UI-автотест.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Приложение открыто на экране авторизации с активными ресурсами тёмной темы. Поле логина доступно для ввода.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Нейтральный текст ContrastSample; синтетический пароль Synthetic123. Выбранный критерий контраста — 4,5:1.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>1. Активировать тёмную тему приложения. 2. Открыть экран авторизации. 3. Ввести ContrastSample в поле логина. 4. Скрыть клавиатуру и проверить отображение и контраст текста.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Введённый текст читаем на фоне поля. Для выбранного критерия QA отношение контраста не ниже 4,5:1.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Текст хранится в поле, но визуально не читается на белой заливке. Отношение контраста текста и фона равно 1,0:1.</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Воспроизведён при пошаговой проверке и UI-автотестом loginFieldHasReadableContrastInNightMode.</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>26.10.2026</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>TC-066; CHK-066</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>docs/evidence/expanded-2026-10-26/BUG-002-dark-auth.png; allure-results.zip</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Успешный вход в тёмной теме проверяется отдельно TC-065. Дефект относится к читаемости введённого текста. Источник выбранного QA-критерия: WCAG 2.2 SC 1.4.3, https://www.w3.org/WAI/WCAG22/Understanding/contrast-minimum.html; проверен 26.10.2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="360" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>BUG-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Подтверждение календаря и времени без изменений сбрасывает сохранённые значения публикации</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Major / значительная</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>P1 / высокий</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Открыт; подтверждён полным UI-прогоном 26.10.2026</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Новости → Редактирование / дата и время</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>1.0.0 (14), debug</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Android 16 / API 36; x86_64; Pixel 6, 1080×2400; en-US; GMT / UTC; debug 1.0.0 (14); AGP 8.12.2 / Gradle 8.13. UI-автотест.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Выполнен вход, создана собственная новость с датой публикации через три дня и временем 23:47.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Собственная новость QA_DIPLOMA_&lt;UUID&gt;; дата для прогона 26.10.2026 — 29.10.2026; время 23:47.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Вариант даты: 1. Открыть редактирование новости. 2. Нажать дату публикации. 3. Не менять выбранные значения, нажать OK. 4. Проверить дату в форме.
+Вариант времени: 1. Заново открыть редактирование исходной новости. 2. Нажать время публикации. 3. Не менять значения, нажать OK. 4. Проверить время в форме.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Диалоги открываются на сохранённых значениях; подтверждение без выбора другой даты или времени сохраняет 29.10.2026 и 23:47.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>В полном прогоне 26.10.2026 дата в форме заменяется на 26.10.2026 вместо 29.10.2026; время заменяется на 19:19 вместо 23:47. После подтверждения без изменения выбора форма содержит непреднамеренные изменения.</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Воспроизведён отдельно для календаря и выбора времени тестами unchangedDatePickerPreservesSavedDate и unchangedTimePickerPreservesSavedTime.</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>26.10.2026</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>TC-084; TC-085; CHK-084; CHK-085</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>docs/evidence/expanded-2026-10-26/BUG-003-date-picker.png; docs/evidence/expanded-2026-10-26/BUG-003-time-picker.png; allure-results.zip</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Оба варианта оформлены одним дефектом и проверены разными сценариями. Значение текущего времени зависит от момента проверки. Непреднамеренная смена значения подтверждена в форме до нажатия Save; поведение сервера после сохранения этим тестом не устанавливается.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="360" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>BUG-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Созданная опубликованная новость исчезает из панели после перехода между разделами</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Critical / критическая</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>P1 / высокий</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Открыт; подтверждён полным UI-прогоном 26.10.2026</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Новости → Панель управления / повторная загрузка</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>1.0.0 (14), debug</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Android 16 / API 36; x86_64; Pixel 6, 1080×2400; en-US; GMT / UTC; debug 1.0.0 (14); AGP 8.12.2 / Gradle 8.13. UI-автотест.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Выполнен вход, доступна панель управления. Лента учебного backend содержит новости с разными датами публикации.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Собственная новость QA_DIPLOMA_&lt;UUID&gt;; дата публикации — текущая дата, время 00:01, Active. До перехода точный заголовок и ID видны в созданной карточке. В итоговом прогоне: заголовок QA_DIPLOMA_8262e8eb-2775-4f66-8f4b-813e7e016e58, зарегистрированный ID 63294.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>1. Открыть Панель управления. 2. Создать собственную новость с текущей датой публикации. 3. Проверить точный заголовок в панели. 4. Через меню перейти в Новости. 5. Снова открыть Панель управления. 6. Дождаться завершения обновления и проверить ту же запись.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Созданная новость остаётся доступна в панели после переходов и повторного чтения данных.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Сразу после сохранения карточка доступна. После перехода Новости → Панель управления точного заголовка нет в загруженном списке.</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Воспроизведён в полном прогоне 26.10.2026 тестом publishedNewsRemainsAfterSectionNavigation; ожидание точного заголовка после обновления завершилось неуспешно.</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>26.10.2026</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>TC-088; CHK-088</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>docs/evidence/expanded-2026-10-26/BUG-004-news-after-navigation.png; allure-results.zip</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Это дефект доступности записи в интерфейсе; удаление записи на backend не установлено. При исследовании наблюдался ответ GET news?pages=1&amp;publishDate=false с 8 элементами и полем pages=203. Клиент заменяет локальную ленту данными полученного ответа; точная серверная семантика поля pages не подтверждена. Для очистки используется только ID собственной записи, зарегистрированный до перехода. После фиксации дефекта собственная запись удалена резервной очисткой по ранее зарегистрированному ID; шаг очистки завершён успешно.</t>
         </is>
       </c>
     </row>

</xml_diff>